<commit_message>
submit: react-select support for Greenhouse, sticky-banner-proof clicks, per-item answers first, resume only into resume fields, emailed verification code asked via Telegram + /ask page, submitted_at only on success
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/referral-tracker.xlsx
+++ b/tracking/referral-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -777,6 +777,67 @@
       </c>
       <c r="N5" s="2" t="inlineStr"/>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Yannic Kilcher</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Chief Technology Officer</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Deepjudge</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>connection at the company</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ykilcher</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Hi Yannic,
+Hope you're well. I saw you're at Deepjudge as a Chief Technology Officer — I've just applied for the
+Machine Learning Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
submit: survive portal re-renders (wait for DOM to settle, re-tag all fields together), stable ids for react-select, exact>prefix>contains option match, never guess a Yes/No, forced click for styled checkboxes, submit pass records its own fill report
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/referral-tracker.xlsx
+++ b/tracking/referral-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -838,6 +838,275 @@
       </c>
       <c r="N6" s="2" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Manish Rathi</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">iOS Guild lead @catawiki | core contributor @fastlane 🚀 </t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Catawiki</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Data Scientist - Machine Learning</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/crazymanish</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Catawiki for the Data Scientist - Machine Learning role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Fabricio Chalub</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Catawiki</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Data Scientist - Machine Learning</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/fcbr</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Catawiki for the Data Scientist - Machine Learning role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Maarten van der Velden</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Catawiki</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Data Scientist - Machine Learning</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/mvandervelden</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Catawiki for the Data Scientist - Machine Learning role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Michal Zygar</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Catawiki</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Data Scientist - Machine Learning</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/mzygar</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Catawiki for the Data Scientist - Machine Learning role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Yannic Kilcher</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Chief Technology Officer</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Deepjudge</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>connection at the company</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ykilcher</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Hi Yannic,
+Hope you're well. I saw you're at Deepjudge as a Chief Technology Officer — I've just applied for the
+Applied AI Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
submit: poll for async typeahead suggestions
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/referral-tracker.xlsx
+++ b/tracking/referral-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1107,6 +1107,431 @@
       </c>
       <c r="N11" s="2" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Prateek Agarwal</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Airwallex</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer (Risk &amp; Payments)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>founder — only if you know them well</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/prateekagwl</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Hi Prateek,
+Hope you're well. I saw you're at Airwallex as a Founder — I've just applied for the
+Senior AI Engineer (Risk &amp; Payments) role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>leon-zhang-awx</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Airwallex</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer (Risk &amp; Payments)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/leon-zhang-awx</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Airwallex for the Senior AI Engineer (Risk &amp; Payments) role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Billy Zou</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Airwallex</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer (Risk &amp; Payments)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/awx-billy-zou</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Airwallex for the Senior AI Engineer (Risk &amp; Payments) role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Able Lv</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Airwallex</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer (Risk &amp; Payments)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/able8</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Airwallex for the Senior AI Engineer (Risk &amp; Payments) role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>David Wheeler</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Staff engineer at @cultureamp </t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Culture Amp</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Senior Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/davidwheeler123</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Culture Amp for the Senior Applied AI Engineer role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Vahid Hallaji</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Culture Amp</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Senior Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/hallaji</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Culture Amp for the Senior Applied AI Engineer role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Rizky</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>I'm a 01X engineer, already halfway to 10X!</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Culture Amp</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Senior Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/itsnotrisky</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Culture Amp for the Senior Applied AI Engineer role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>James Telfer</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Culture Amp</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Senior Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jamestelfer</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Culture Amp for the Senior Applied AI Engineer role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Workday: social sign-in chooser ('Sign in with email'), sign-in/create error text captured, create-then-bounce treated as email verification (asked on Telegram)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/referral-tracker.xlsx
+++ b/tracking/referral-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1924,6 +1924,214 @@
       </c>
       <c r="N26" s="2" t="inlineStr"/>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>rohansav</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Reflectionai</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Member of Technical Staff - Pre-Training</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/rohansav</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Reflectionai for the Member of Technical Staff - Pre-Training role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Ralph J. Recto</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Reflectionai</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Member of Technical Staff - Pre-Training</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/ralphrecto</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Reflectionai for the Member of Technical Staff - Pre-Training role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Cody</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Reflectionai</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Member of Technical Staff - Pre-Training</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/unsleepy22</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Reflectionai for the Member of Technical Staff - Pre-Training role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Adrien Barbaresi</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Reflectionai</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Member of Technical Staff - Pre-Training</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/adbar</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Reflectionai for the Member of Technical Staff - Pre-Training role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
applications: hooks.py and replay.json for every application; new Berkadia, Capital One, Just Eat Takeaway folders; referral tracker
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/referral-tracker.xlsx
+++ b/tracking/referral-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2132,6 +2132,754 @@
       </c>
       <c r="N30" s="2" t="inlineStr"/>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Aashcharya Gorakh</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/aashcharya-gorakh-a764a2287</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Hi Aashcharya,
+Hope you're well. I saw you're at MongoDB as a Software Engineer Intern — I've just applied for the
+Senior Data Scientist role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Caitlyn Kupski</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Senior Technical Recruiter</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>recruiter</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/caitlynkelly</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Hi Caitlyn,
+Hope you're well. I saw you're at MongoDB as a Senior Technical Recruiter — I've just applied for the
+Senior Data Scientist role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Agustin Bettati</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/AgustinBettati</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring MongoDB for the Senior Data Scientist role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>A. Jesse Jiryu Davis</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Senior Staff Research Engineer in the MongoDB Distributed Sy</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/ajdavis</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring MongoDB for the Senior Data Scientist role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Avinash Pathak</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Nvidia</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Senior Research Scientist for Generative AI</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/avipathak99</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Hi Avinash,
+Hope you're well. I saw you're at Nvidia as a Senior AI Engineer — I've just applied for the
+Senior Research Scientist for Generative AI role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Shubham Pachori</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Sr. Applied Scientist</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Nvidia</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Senior Research Scientist for Generative AI</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/shubhampachori</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Hi Shubham,
+Hope you're well. I saw you're at Nvidia as a Sr. Applied Scientist — I've just applied for the
+Senior Research Scientist for Generative AI role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Raviraj Joshi</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Nvidia</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Senior Research Scientist for Generative AI</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ravirajoshi</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Hi Raviraj,
+Hope you're well. I saw you're at Nvidia as a Senior Data Scientist — I've just applied for the
+Senior Research Scientist for Generative AI role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Ivan Sorokin</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Reinforcement Learning -&gt; Speech Recognition -&gt; Natural Lang</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Nvidia</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Senior Research Scientist for Generative AI</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/1ytic</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Nvidia for the Senior Research Scientist for Generative AI role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Avinash D</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Lead AI Engineer</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Capital One Careers</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>AI Engineer 4 (Gen AI Platform Services: Agentic AI, Agent Guardrails, Agent Evaluation, Agent Memory) at Capital One</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/avinash-d26</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>Hi Avinash,
+Hope you're well. I saw you're at Capital One Careers as a Lead AI Engineer — I've just applied for the
+AI Engineer 4 (Gen AI Platform Services: Agentic AI, Agent Guardrails, Agent Evaluation, Agent Memory) at Capital One role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Kalanand Mishra, PhD</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Director, Applied AI - AI Foundations</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Capital One Careers</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>AI Engineer 4 (Gen AI Platform Services: Agentic AI, Agent Guardrails, Agent Evaluation, Agent Memory) at Capital One</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>founder — only if you know them well</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kalanand</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Hi Kalanand,
+Hope you're well. I saw you're at Capital One Careers as a Director, Applied AI - AI Foundations — I've just applied for the
+AI Engineer 4 (Gen AI Platform Services: Agentic AI, Agent Guardrails, Agent Evaluation, Agent Memory) at Capital One role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Shashank Karnawat</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Senior Business Manager</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Capital One Careers</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>AI Engineer 4 (Gen AI Platform Services: Agentic AI, Agent Guardrails, Agent Evaluation, Agent Memory) at Capital One</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>connection at the company</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/shashankkarnawat</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Hi Shashank,
+Hope you're well. I saw you're at Capital One Careers as a Senior Business Manager — I've just applied for the
+AI Engineer 4 (Gen AI Platform Services: Agentic AI, Agent Guardrails, Agent Evaluation, Agent Memory) at Capital One role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Andreas Hechenberger</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Takeaway</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Senior Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/hechi</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Takeaway for the Senior Forward Deployed Engineer role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Emre Piskin</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Software Development Team Lead</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Takeaway</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Senior Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/pemre</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Takeaway for the Senior Forward Deployed Engineer role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Review list: "Needs you now" for filings waiting on him; sent cards protected
- ask.py: a question records its job and deadline; the Telegram message is a card (job,
  question, deadline, link); open_asks() for the review list
- review list: "Needs you now — a filing is waiting" at the top, answer box and Send on the
  list; "Sent? — check your email" for unconfirmed cards (they had no section)
- dedupe: a card that was or may have been sent (submitted / unconfirmed / submitting / a
  recorded press) is never removed — it had deleted the unconfirmed OpenAI card; superseded
  ranks last; the OpenAI card restored
- filing refuses a job whose record shows a submitted or unconfirmed attempt

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/referral-tracker.xlsx
+++ b/tracking/referral-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4120,6 +4120,372 @@
       </c>
       <c r="N65" s="2" t="inlineStr"/>
     </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>BHASKAR KURASALA</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Sr. Gen AI Engineer (FDE)</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Turing</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Senior Research Engineer, SWE</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/bhaskar-kurasala-ai-engineer</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>Hi BHASKAR,
+Hope you're well. I saw you're at Turing as a Sr. Gen AI Engineer (FDE) — I've just applied for the
+Senior Research Engineer, SWE role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Umang Kumar Sinha</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Senior Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Turing</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Senior Research Engineer, SWE</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/umangkrsinha</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr"/>
+      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>Hi Umang,
+Hope you're well. I saw you're at Turing as a Senior Machine Learning Engineer — I've just applied for the
+Senior Research Engineer, SWE role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>kalyan sekhar gali</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Turing</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Senior Research Engineer, SWE</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kalyan-sekhar</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>Hi kalyan sekhar,
+Hope you're well. I saw you're at Turing as a Machine Learning Engineer — I've just applied for the
+Senior Research Engineer, SWE role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>BHASKAR KURASALA</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Sr. Gen AI Engineer (FDE)</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Turing</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Senior Research Engineer, Frontier Data</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/bhaskar-kurasala-ai-engineer</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr"/>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>Hi BHASKAR,
+Hope you're well. I saw you're at Turing as a Sr. Gen AI Engineer (FDE) — I've just applied for the
+Senior Research Engineer, Frontier Data role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Umang Kumar Sinha</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Senior Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Turing</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Senior Research Engineer, Frontier Data</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/umangkrsinha</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>Hi Umang,
+Hope you're well. I saw you're at Turing as a Senior Machine Learning Engineer — I've just applied for the
+Senior Research Engineer, Frontier Data role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>kalyan sekhar gali</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Turing</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Senior Research Engineer, Frontier Data</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kalyan-sekhar</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="2" t="inlineStr"/>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>Hi kalyan sekhar,
+Hope you're well. I saw you're at Turing as a Machine Learning Engineer — I've just applied for the
+Senior Research Engineer, Frontier Data role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Review list: Submitted as a dated table, newest first (date, company, role, filed / by hand)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/referral-tracker.xlsx
+++ b/tracking/referral-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N71"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4486,6 +4486,345 @@
       </c>
       <c r="N71" s="2" t="inlineStr"/>
     </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Andreas Hechenberger</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Takeaway</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/hechi</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Takeaway for the Senior Data Scientist role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Emre Piskin</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Software Development Team Lead</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Takeaway</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/pemre</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr"/>
+      <c r="J73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr"/>
+      <c r="L73" s="2" t="inlineStr"/>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Takeaway for the Senior Data Scientist role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Sameer Khurana</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Member of Technical Staff</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Exa</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>senior engineer</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sameer-khurana-9a40b772</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>Hi Sameer,
+Hope you're well. I saw you're at Exa as a Member of Technical Staff — I've just applied for the
+Forward Deployed Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Aparna Kadiyala</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Exa</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/aparna-kadiyala526</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr"/>
+      <c r="L75" s="2" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>Hi Aparna,
+Hope you're well. I saw you're at Exa as a Software Engineer — I've just applied for the
+Forward Deployed Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Neeraj Soni</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Associate Software Developer</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Exa</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/neerajsoni11</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>Hi Neeraj,
+Hope you're well. I saw you're at Exa as a Associate Software Developer — I've just applied for the
+Forward Deployed Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Sergey Kuleshov</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Exa</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/svyatogor</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr"/>
+      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Exa for the Forward Deployed Engineer role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Docs: the old see/map/act plans removed; docs/form-agent.md describes what is built
Exploring, the record and resuming, filing and every Submit outcome, techniques per control,
dates, questions during filing, the review list, the safety rules, files, known limits.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/referral-tracker.xlsx
+++ b/tracking/referral-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N77"/>
+  <dimension ref="A1:N81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4825,6 +4825,241 @@
       </c>
       <c r="N77" s="2" t="inlineStr"/>
     </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Harsh Agarwal</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer 4</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Research Engineer</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/harsh-aga</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>Hi Harsh,
+Hope you're well. I saw you're at Adobe as a Machine Learning Engineer 4 — I've just applied for the
+Research Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Nikhil Pentapalli</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Senior Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Research Engineer</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nikhilpentapalli</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr"/>
+      <c r="L79" s="2" t="inlineStr"/>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>Hi Nikhil,
+Hope you're well. I saw you're at Adobe as a Senior Machine Learning Engineer — I've just applied for the
+Research Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Mohit Chawla</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer 4</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Research Engineer</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mohitchawla16</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>Hi Mohit,
+Hope you're well. I saw you're at Adobe as a Machine Learning Engineer 4 — I've just applied for the
+Research Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Mariia Lukianets</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Research Engineer</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/3ch023</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr"/>
+      <c r="K81" s="2" t="inlineStr"/>
+      <c r="L81" s="2" t="inlineStr"/>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Adobe for the Research Engineer role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
CLI and docs reviewed: submit <slug> files one job, dryrun added; stale passages rewritten
- jobpilot: `submit <slug>` files that one approved job (it used to ignore the slug and file
  everything); `dryrun <slug>` stops before Submit; `link` also prints /questions; help text
  for explore (resumes, --fresh) and the Claude-usage note
- README: the scan diagram (screen stage, form agent, card), the Telegram outcomes (captcha,
  code-needed, unconfirmed), the Workday paragraph, filing's Claude use, conflict questions,
  the command list
- agents/README: only the three CLI agents that exist; the form agent lives in explore_agentic
- docs/form-agent.md: the commands
- tracking/referral-tracker.xlsx: referral targets found after today's submissions

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/referral-tracker.xlsx
+++ b/tracking/referral-tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N81"/>
+  <dimension ref="A1:N85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5060,6 +5060,241 @@
       </c>
       <c r="N81" s="2" t="inlineStr"/>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Harsh Agarwal</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer 4</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Sr. Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/harsh-aga</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>Hi Harsh,
+Hope you're well. I saw you're at Adobe as a Machine Learning Engineer 4 — I've just applied for the
+Sr. Applied AI Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Nikhil Pentapalli</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Senior Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Sr. Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nikhilpentapalli</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr"/>
+      <c r="K83" s="2" t="inlineStr"/>
+      <c r="L83" s="2" t="inlineStr"/>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>Hi Nikhil,
+Hope you're well. I saw you're at Adobe as a Senior Machine Learning Engineer — I've just applied for the
+Sr. Applied AI Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Mohit Chawla</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer 4</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Sr. Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>1st-degree</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>works in your field</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mohitchawla16</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr"/>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>Hi Mohit,
+Hope you're well. I saw you're at Adobe as a Machine Learning Engineer 4 — I've just applied for the
+Sr. Applied AI Engineer role there and wondered if you'd be open to referring me internally.
+Quick context: ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI. Most relevant to this role, I built an evaluation harness with a cell-level F1 grader that benchmarks our agent fleet at 86% exact-pass,
+and Phi-3 Vision on vLLM at 20 ms median latency in production.
+No pressure at all if it's not something you're comfortable doing, or if you
+don't know the team. If it helps, I can send my resume and a two-line summary
+you could paste straight into the referral form.
+Thanks either way,
+Sunil</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Mariia Lukianets</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Sr. Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>cold (GitHub)</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>engineer on public repos</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/3ch023</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>To Contact</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr"/>
+      <c r="K85" s="2" t="inlineStr"/>
+      <c r="L85" s="2" t="inlineStr"/>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>Hi — ML engineer here (ex-Amazon Applied Scientist, M.Tech in AI from IIT Jodhpur, ~5 years building production AI). I'm exploring Adobe for the Sr. Applied AI Engineer role and would value connecting with someone doing this work there.</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>